<commit_message>
feat(excel): support struct column expansion
Add columns parser projection support across IR validation, CSV/XLSX input readers, and generated Excel templates. Regenerate showcase workbooks and generated outputs, including root-type notes for expanded cells.
</commit_message>
<xml_diff>
--- a/examples/showcase/data/Complex.xlsx
+++ b/examples/showcase/data/Complex.xlsx
@@ -188,9 +188,312 @@
           </rPr>
           <t xml:space="preserve">
 Field: value
-Type: union&lt;EventCondition&gt;
+Type: union&lt;EventCondition&gt; tag
+Root field: value
+Root type: union&lt;EventCondition&gt;
 Parser: tagged_columns
 Column: type</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.level
+Type: ref&lt;LevelExp.level&gt;
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns
+Column: level</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.quest_id
+Type: ref&lt;Quest.id&gt;
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns
+Column: quest_id</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.item_id
+Type: ref&lt;Item.id&gt;
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns
+Column: item_id</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.count
+Type: i32
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns
+Column: count</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.condition_group_id
+Type: ref&lt;ComplexConditionGroup.id&gt;
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns
+Column: condition_group_id</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns</t>
         </r>
       </text>
     </comment>
@@ -226,9 +529,312 @@
           </rPr>
           <t xml:space="preserve">
 Field: value
-Type: union&lt;EventCondition&gt;
+Type: union&lt;EventCondition&gt; tag
+Root field: value
+Root type: union&lt;EventCondition&gt;
 Parser: tagged_columns
 Column: type</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.level
+Type: ref&lt;LevelExp.level&gt;
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns
+Column: level</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.quest_id
+Type: ref&lt;Quest.id&gt;
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns
+Column: quest_id</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.item_id
+Type: ref&lt;Item.id&gt;
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns
+Column: item_id</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.count
+Type: i32
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns
+Column: count</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.condition_group_id
+Type: ref&lt;ComplexConditionGroup.id&gt;
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns
+Column: condition_group_id</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;EventCondition&gt;
+Parser: tagged_columns</t>
         </r>
       </text>
     </comment>
@@ -264,9 +870,422 @@
           </rPr>
           <t xml:space="preserve">
 Field: value
-Type: union&lt;RewardAction&gt;
+Type: union&lt;RewardAction&gt; tag
+Root field: value
+Root type: union&lt;RewardAction&gt;
 Parser: tagged_columns
 Column: type</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.item_id
+Type: ref&lt;Item.id&gt;
+Root field: value
+Root type: union&lt;RewardAction&gt;
+Parser: tagged_columns
+Column: item_id</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.count
+Type: i32
+Root field: value
+Root type: union&lt;RewardAction&gt;
+Parser: tagged_columns
+Column: count</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.buff_id
+Type: ref&lt;Buff.id&gt;
+Root field: value
+Root type: union&lt;RewardAction&gt;
+Parser: tagged_columns
+Column: buff_id</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.duration
+Type: f32
+Root field: value
+Root type: union&lt;RewardAction&gt;
+Parser: tagged_columns
+Column: duration</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.stage_id
+Type: ref&lt;Stage.id&gt;
+Root field: value
+Root type: union&lt;RewardAction&gt;
+Parser: tagged_columns
+Column: stage_id</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.mail_id
+Type: ref&lt;MailTemplate.id&gt;
+Root field: value
+Root type: union&lt;RewardAction&gt;
+Parser: tagged_columns
+Column: mail_id</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L2" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Field: value.action_group_id
+Type: ref&lt;ComplexActionGroup.id&gt;
+Root field: value
+Root type: union&lt;RewardAction&gt;
+Parser: tagged_columns
+Column: action_group_id</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;RewardAction&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;RewardAction&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;RewardAction&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;RewardAction&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;RewardAction&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;RewardAction&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;RewardAction&gt;
+Parser: tagged_columns</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L4" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sora:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Root field: value
+Root type: union&lt;RewardAction&gt;
+Parser: tagged_columns</t>
         </r>
       </text>
     </comment>
@@ -668,7 +1687,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -701,13 +1720,30 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF0F172A"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0F172A"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="8"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -756,6 +1792,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDF7EE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -784,7 +1826,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -806,6 +1848,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1527,22 +2581,22 @@
       <c r="D2" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="9" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1559,22 +2613,22 @@
       <c r="D3" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="10" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1591,22 +2645,22 @@
       <c r="D4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="J4" s="10" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1623,22 +2677,22 @@
       <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J5" s="5" t="s">
+      <c r="E5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="10" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1651,16 +2705,16 @@
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5" t="s">
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="J6" s="5"/>
+      <c r="J6" s="10"/>
     </row>
     <row r="7" spans="1:10" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
@@ -1669,14 +2723,14 @@
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="11"/>
     </row>
     <row r="8" spans="1:10">
       <c r="B8" s="5" t="s">
@@ -1838,22 +2892,22 @@
       <c r="C2" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="9" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1867,22 +2921,22 @@
       <c r="C3" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="10" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1896,22 +2950,22 @@
       <c r="C4" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="10" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1925,22 +2979,22 @@
       <c r="C5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="5" t="s">
+      <c r="D5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="10" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1952,16 +3006,16 @@
         <v>26</v>
       </c>
       <c r="C6" s="5"/>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5" t="s">
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="I6" s="5"/>
+      <c r="I6" s="10"/>
     </row>
     <row r="7" spans="1:10" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
@@ -1969,14 +3023,14 @@
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
     </row>
     <row r="8" spans="1:10">
       <c r="B8" s="5" t="s">
@@ -2248,28 +3302,28 @@
       <c r="D2" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="9" t="s">
         <v>105</v>
       </c>
     </row>
@@ -2286,28 +3340,28 @@
       <c r="D3" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="K3" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="L3" s="10" t="s">
         <v>105</v>
       </c>
     </row>
@@ -2324,28 +3378,28 @@
       <c r="D4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="J4" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="K4" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="L4" s="10" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2362,28 +3416,28 @@
       <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="L5" s="5" t="s">
+      <c r="E5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="10" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2396,18 +3450,18 @@
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5" t="s">
+      <c r="F6" s="10"/>
+      <c r="G6" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10"/>
     </row>
     <row r="7" spans="1:12" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
@@ -2416,16 +3470,16 @@
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="11"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
     </row>
     <row r="8" spans="1:12">
       <c r="B8" s="5" t="s">

</xml_diff>